<commit_message>
pubgen: thread overset narrative text, parse pub_office for BRS cover, and style hf-brs with Raleway #f68839
- Auto-thread narrative text frames overflowing page bottom to continuation pages and tighten frame bounds
- Force GXX graphic/chart sheets in BPS BRS to start on a new page
- Parse pub_office / kantorpublikasi from Excel cover sheet and prioritize next to BPS cover logo
- Configure hf-brs preset with Raleway font and #f68839 color, applying footer-only folio and metadata
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/brs/ntp202610.xlsx
+++ b/plan/pubgen/samples/brs/ntp202610.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft-pubgen\plan\pubgen\samples\brs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7732774E-A9E3-4BC8-8412-673B6682515E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFE2EA1-141A-4A8C-8CAF-4C4709191BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4095" yWindow="1275" windowWidth="19935" windowHeight="9720" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4095" yWindow="1275" windowWidth="19935" windowHeight="9720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COV" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="186">
   <si>
     <t>Sep'25</t>
   </si>
@@ -587,6 +587,12 @@
   </si>
   <si>
     <t>line</t>
+  </si>
+  <si>
+    <t>BADAN PUSAT STATISTIK PROVINSI JAWA BARAT</t>
+  </si>
+  <si>
+    <t>pub_office</t>
   </si>
 </sst>
 </file>
@@ -1040,7 +1046,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4959391-8906-46B1-88E9-2AFBA1159CFD}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -1081,81 +1087,89 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" t="s">
-        <v>61</v>
+        <v>185</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="5">
-        <v>46266</v>
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46266</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
-        <v>177</v>
+        <v>63</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>178</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B12" t="s">
-        <v>171</v>
+        <v>169</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>173</v>
       </c>
     </row>

</xml_diff>